<commit_message>
Add DOI and stabilize reproducible outputs
</commit_message>
<xml_diff>
--- a/outputs/tables/supplementary_tables.xlsx
+++ b/outputs/tables/supplementary_tables.xlsx
@@ -4905,13 +4905,13 @@
         <v>5000</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.08158368326334731</v>
+        <v>0.1125774845030993</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.08158368326334731</v>
+        <v>0.1125774845030993</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.7482</v>
+        <v>0.8972</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
@@ -4947,13 +4947,13 @@
         <v>5000</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>0.1339732053589282</v>
+        <v>0.1355728854229154</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>0.1237752449510097</v>
+        <v>0.1355728854229154</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0.675</v>
+        <v>0.8596</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
@@ -9619,7 +9619,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit MetaCyc fermentation pathway producing butanoate; retained as core butyrate/butanoate encoded-potential feature. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=CENTFERM-PWY&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit MetaCyc fermentation pathway producing butanoate; retained as core butyrate/butanoate encoded-potential feature. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=CENTFERM-PWY&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -9629,7 +9629,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -9666,7 +9666,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit MetaCyc fermentation pathway from acetyl-CoA to butanoate; retained as core butyrate/butanoate encoded-potential feature. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=PWY-5676&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit MetaCyc fermentation pathway from acetyl-CoA to butanoate; retained as core butyrate/butanoate encoded-potential feature. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=PWY-5676&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -9676,7 +9676,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -9713,7 +9713,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit succinate-to-butanoate fermentation pathway; assigned to butyrate/butanoate submodule by terminal product. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5677&amp;orgids=http%27&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit succinate-to-butanoate fermentation pathway; assigned to butyrate/butanoate submodule by terminal product. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5677&amp;orgids=http%27&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -9723,7 +9723,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -9760,7 +9760,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit amino-acid fermentation pathway producing butanoate and acetate; assigned to butyrate/butanoate submodule by terminal butanoate product and not duplicated in acetate submodule. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=P163-PWY&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit amino-acid fermentation pathway producing butanoate and acetate; assigned to butyrate/butanoate submodule by terminal butanoate product and not duplicated in acetate submodule. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=P163-PWY&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -9770,7 +9770,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -9807,7 +9807,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit pyruvate fermentation pathway producing acetate and lactate; retained in acetate submodule and duplicated in lactate/succinate submodule as a planned multi-product overlap. BioCyc/MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=P41-PWY&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit pyruvate fermentation pathway producing acetate and lactate; retained in acetate submodule and duplicated in lactate/succinate submodule as a planned multi-product overlap. BioCyc/MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=P41-PWY&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -9817,7 +9817,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -9854,7 +9854,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit pyruvate fermentation pathway producing acetate and lactate; retained in acetate submodule and duplicated in lactate/succinate submodule as a planned multi-product overlap. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5100&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit pyruvate fermentation pathway producing acetate and lactate; retained in acetate submodule and duplicated in lactate/succinate submodule as a planned multi-product overlap. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5100&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -9901,7 +9901,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. BioCyc/MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=P41-PWY&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. BioCyc/MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=P41-PWY&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -9911,7 +9911,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -9948,7 +9948,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5100&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5100&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -9995,7 +9995,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 comparator: retained as non-fermentation amino-acid biosynthesis comparator; not interpreted as measured indole production. MetaCyc database rationale only; broad superpathway noted. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparator: retained as non-fermentation amino-acid biosynthesis comparator; not interpreted as measured indole production. MetaCyc database rationale only; broad superpathway noted. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 comparator: retained as non-fermentation amino-acid biosynthesis comparator; not interpreted as measured indole production. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparator: retained as non-fermentation amino-acid biosynthesis comparator; not interpreted as measured indole production. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -10052,7 +10052,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10089,7 +10089,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 negative-control comparator: cell-envelope/lipid-A biosynthesis module, not SCFA fermentation. Broad superpathway retained only as comparator. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparison module: cell-envelope/lipid-A biosynthesis module, not SCFA fermentation. Broad superpathway retained only as comparator. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -10099,7 +10099,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10136,7 +10136,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 negative-control comparator: lipid A-core biosynthesis module, not SCFA fermentation. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparison module: lipid A-core biosynthesis module, not SCFA fermentation. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -10146,7 +10146,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10183,7 +10183,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 negative-control comparator: lipopolysaccharide biosynthesis module, not SCFA fermentation. Broad superpathway retained only as comparator. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparison module: lipopolysaccharide biosynthesis module, not SCFA fermentation. Broad superpathway retained only as comparator. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -10193,7 +10193,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10230,7 +10230,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 exploratory comparator: bile-acid transformation pathway retained outside the primary hypothesis. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition exploratory comparator: bile-acid transformation pathway retained outside the primary hypothesis. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -10240,7 +10240,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10277,7 +10277,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit MetaCyc fermentation pathway producing butanoate; retained as core butyrate/butanoate encoded-potential feature. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=CENTFERM-PWY&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit MetaCyc fermentation pathway producing butanoate; retained as core butyrate/butanoate encoded-potential feature. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=CENTFERM-PWY&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -10287,7 +10287,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10324,7 +10324,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit MetaCyc fermentation pathway from acetyl-CoA to butanoate; retained as core butyrate/butanoate encoded-potential feature. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=PWY-5676&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit MetaCyc fermentation pathway from acetyl-CoA to butanoate; retained as core butyrate/butanoate encoded-potential feature. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=PWY-5676&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10371,7 +10371,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit succinate-to-butanoate fermentation pathway; assigned to butyrate/butanoate submodule by terminal product. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5677&amp;orgids=http%27&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit succinate-to-butanoate fermentation pathway; assigned to butyrate/butanoate submodule by terminal product. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5677&amp;orgids=http%27&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -10381,7 +10381,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10418,7 +10418,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit amino-acid fermentation pathway producing butanoate and acetate; assigned to butyrate/butanoate submodule by terminal butanoate product and not duplicated in acetate submodule. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=P163-PWY&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit amino-acid fermentation pathway producing butanoate and acetate; assigned to butyrate/butanoate submodule by terminal butanoate product and not duplicated in acetate submodule. BioCyc/MetaCyc: https://biocyc.org/META/NEW-IMAGE?object=P163-PWY&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10465,7 +10465,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit pyruvate fermentation pathway producing acetate and lactate; retained in acetate submodule and duplicated in lactate/succinate submodule as a planned multi-product overlap. BioCyc/MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=P41-PWY&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit pyruvate fermentation pathway producing acetate and lactate; retained in acetate submodule and duplicated in lactate/succinate submodule as a planned multi-product overlap. BioCyc/MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=P41-PWY&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -10475,7 +10475,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10512,7 +10512,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit pyruvate fermentation pathway producing acetate and lactate; retained in acetate submodule and duplicated in lactate/succinate submodule as a planned multi-product overlap. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5100&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit pyruvate fermentation pathway producing acetate and lactate; retained in acetate submodule and duplicated in lactate/succinate submodule as a planned multi-product overlap. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5100&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -10522,7 +10522,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10559,7 +10559,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 expanded member: explicit fermentation pathway with acetate and lactate among products; expanded only because substrate and product mix are broader than pyruvate core. MetaCyc pathway name from HUMAnN/MetaCyc seed table.</t>
+          <t>Finalised analysis definition expanded member: explicit fermentation pathway with acetate and lactate among products; expanded only because substrate and product mix are broader than pyruvate core. MetaCyc pathway name from HUMAnN/MetaCyc seed table.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -10569,7 +10569,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10606,7 +10606,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 expanded member: explicit lactate fermentation pathway with acetate as a product; expanded only because terminal product is propanoate rather than acetate/butanoate alone. MetaCyc: https://metacyc.org/META/NEW-IMAGE?object=PWY-8086&amp;redirect=T&amp;type=NIL</t>
+          <t>Finalised analysis definition expanded member: explicit lactate fermentation pathway with acetate as a product; expanded only because terminal product is propanoate rather than acetate/butanoate alone. MetaCyc: https://metacyc.org/META/NEW-IMAGE?object=PWY-8086&amp;redirect=T&amp;type=NIL</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -10616,7 +10616,7 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10653,7 +10653,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. BioCyc/MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=P41-PWY&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. BioCyc/MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=P41-PWY&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -10663,7 +10663,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10700,7 +10700,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Locked v1: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5100&amp;type=PATHWAY</t>
+          <t>Finalised analysis definition: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. MetaCyc: https://vm-trypanocyc.toulouse.inra.fr/META/NEW-IMAGE?object=PWY-5100&amp;type=PATHWAY</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10747,7 +10747,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 expanded member: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. MetaCyc pathway name from HUMAnN/MetaCyc seed table.</t>
+          <t>Finalised analysis definition expanded member: explicit lactate-producing fermentation pathway; planned overlap with acetate submodule because the pathway produces both acetate and lactate. MetaCyc pathway name from HUMAnN/MetaCyc seed table.</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -10757,7 +10757,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10794,7 +10794,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 expanded member: explicit lactate-consuming/propanoate-acetate fermentation pathway retained in lactate/succinate family as lactate-fermentation encoded potential. MetaCyc: https://metacyc.org/META/NEW-IMAGE?object=PWY-8086&amp;redirect=T&amp;type=NIL</t>
+          <t>Finalised analysis definition expanded member: explicit lactate-consuming/propanoate-acetate fermentation pathway retained in lactate/succinate family as lactate-fermentation encoded potential. MetaCyc: https://metacyc.org/META/NEW-IMAGE?object=PWY-8086&amp;redirect=T&amp;type=NIL</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -10804,7 +10804,7 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10841,7 +10841,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 comparator: retained as non-fermentation amino-acid biosynthesis comparator; not interpreted as measured indole production. MetaCyc database rationale only; broad superpathway noted. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparator: retained as non-fermentation amino-acid biosynthesis comparator; not interpreted as measured indole production. MetaCyc database rationale only; broad superpathway noted. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10888,7 +10888,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 comparator: retained as non-fermentation amino-acid biosynthesis comparator; not interpreted as measured indole production. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparator: retained as non-fermentation amino-acid biosynthesis comparator; not interpreted as measured indole production. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -10898,7 +10898,7 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10935,7 +10935,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 negative-control comparator: cell-envelope/lipid-A biosynthesis module, not SCFA fermentation. Broad superpathway retained only as comparator. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparison module: cell-envelope/lipid-A biosynthesis module, not SCFA fermentation. Broad superpathway retained only as comparator. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -10945,7 +10945,7 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -10982,7 +10982,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 negative-control comparator: lipid A-core biosynthesis module, not SCFA fermentation. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparison module: lipid A-core biosynthesis module, not SCFA fermentation. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11029,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 negative-control comparator: lipopolysaccharide biosynthesis module, not SCFA fermentation. Broad superpathway retained only as comparator. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition comparison module: lipopolysaccharide biosynthesis module, not SCFA fermentation. Broad superpathway retained only as comparator. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 expanded negative-control comparator: cell-envelope antigen biosynthesis retained only in expanded comparator, not SCFA fermentation. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition expanded comparison module: cell-envelope antigen biosynthesis retained only in expanded comparator, not SCFA fermentation. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -11086,7 +11086,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -11123,7 +11123,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Locked v1 exploratory comparator: bile-acid transformation pathway retained outside the primary hypothesis. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
+          <t>Finalised analysis definition exploratory comparator: bile-acid transformation pathway retained outside the primary hypothesis. MetaCyc overview: https://metacyc.org/MetaCycUserGuide.shtml</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -11133,7 +11133,7 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>locked</t>
+          <t>finalised</t>
         </is>
       </c>
     </row>
@@ -15446,7 +15446,7 @@
         <v>5000</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.23475304939</v>
+        <v>0.235152969406</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>0.000199960007998</v>

</xml_diff>

<commit_message>
Synchronize submission figure reproducibility
</commit_message>
<xml_diff>
--- a/outputs/tables/supplementary_tables.xlsx
+++ b/outputs/tables/supplementary_tables.xlsx
@@ -7,62 +7,62 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 1 Cohort screening" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 2 Module definitions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 3 Member availability" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 4 Scoring formula" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 5 Statistical settings" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 6 Score sensitivity" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 7 NAFLD covariates" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 8 Endpoint hierarchy" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 9 CHB effects" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 10 CHB expanded" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 11 CHB pathway members" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 12 CHB leave-one-out" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 13 CHB matched sets" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 14 NAFLD effects" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 15 NAFLD pathways" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 16 NAFLD leave-one-out" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 17 NAFLD matched sets" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 18 Cirrhosis effects" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 19 Cirrhosis pathways" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 20 STORMS checklist" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 21 STROBE checklist" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 22 NAFLD technical" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 23 CHB pathway detection" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 24 Log-ratio sensitivity" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 25 Matched set diagnostics" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp 26 Unmapped fractions" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1 Cohort screening" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2 Module definitions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S3 Pathway availability" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S4 Scoring formula" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S5 Statistical methods" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S6 Score sensitivity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S7 NAFLD metadata" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S8 Analysis hierarchy" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S9 CHB effects" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S10 CHB expanded" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S11 CHB pathways" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S12 CHB leave-one-out" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S13 CHB matched sets" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S14 NAFLD effects" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S15 NAFLD pathways" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S16 NAFLD leave-one-out" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S17 NAFLD matched sets" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S18 Cirrhosis effects" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S19 Cirrhosis pathways" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S20 STORMS checklist" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S21 STROBE checklist" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S22 NAFLD technical" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S23 CHB detection" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S24 Log-ratio sensitivity" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S25 Matched diagnostics" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S26 Unmapped fractions" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Table index'!$A$1:$B$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Supp 1 Cohort screening'!$A$1:$D$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Supp 2 Module definitions'!$A$1:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Supp 3 Member availability'!$A$1:$G$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Supp 4 Scoring formula'!$A$1:$B$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Supp 5 Statistical settings'!$A$1:$B$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Supp 6 Score sensitivity'!$A$1:$J$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Supp 7 NAFLD covariates'!$A$1:$F$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Supp 8 Endpoint hierarchy'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Supp 9 CHB effects'!$A$1:$S$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Supp 10 CHB expanded'!$A$1:$S$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Supp 11 CHB pathway members'!$A$1:$O$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Supp 12 CHB leave-one-out'!$A$1:$H$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Supp 13 CHB matched sets'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Supp 14 NAFLD effects'!$A$1:$Y$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Supp 15 NAFLD pathways'!$A$1:$O$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Supp 16 NAFLD leave-one-out'!$A$1:$H$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Supp 17 NAFLD matched sets'!$A$1:$J$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Supp 18 Cirrhosis effects'!$A$1:$Y$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Supp 19 Cirrhosis pathways'!$A$1:$O$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Supp 20 STORMS checklist'!$A$1:$C$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Supp 21 STROBE checklist'!$A$1:$C$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Supp 22 NAFLD technical'!$A$1:$O$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Supp 23 CHB pathway detection'!$A$1:$M$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'Supp 24 Log-ratio sensitivity'!$A$1:$L$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'Supp 25 Matched set diagnostics'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Supp 26 Unmapped fractions'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Table S1 Cohort screening'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Table S2 Module definitions'!$A$1:$I$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Table S3 Pathway availability'!$A$1:$G$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Table S4 Scoring formula'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Table S5 Statistical methods'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Table S6 Score sensitivity'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Table S7 NAFLD metadata'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Table S8 Analysis hierarchy'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Table S9 CHB effects'!$A$1:$S$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Table S10 CHB expanded'!$A$1:$S$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Table S11 CHB pathways'!$A$1:$O$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Table S12 CHB leave-one-out'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Table S13 CHB matched sets'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Table S14 NAFLD effects'!$A$1:$Y$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Table S15 NAFLD pathways'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Table S16 NAFLD leave-one-out'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Table S17 NAFLD matched sets'!$A$1:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Table S18 Cirrhosis effects'!$A$1:$Y$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Table S19 Cirrhosis pathways'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Table S20 STORMS checklist'!$A$1:$C$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Table S21 STROBE checklist'!$A$1:$C$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Table S22 NAFLD technical'!$A$1:$O$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Table S23 CHB detection'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'Table S24 Log-ratio sensitivity'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'Table S25 Matched diagnostics'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Table S26 Unmapped fractions'!$A$1:$K$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>

</xml_diff>